<commit_message>
se agrega flujo de compra
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ing. Gorgona\IdeaProjects\bon-bonite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71AC9B0-0CA0-4418-9625-E487D5129944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0639D33B-0095-47DE-977B-9BD5C4C7A325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{B34893C1-2C1C-4B7A-90BE-5673413F01AD}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>https://www.bon-bonite.com/</t>
   </si>
@@ -98,13 +98,43 @@
   </si>
   <si>
     <t>Disponibles</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>Bota en carnaza moca</t>
+  </si>
+  <si>
+    <t>Talla</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>Celular</t>
+  </si>
+  <si>
+    <t>3003350739</t>
+  </si>
+  <si>
+    <t>Direccion</t>
+  </si>
+  <si>
+    <t>TV 60 CL 114 A - 56</t>
+  </si>
+  <si>
+    <t>Ciudad</t>
+  </si>
+  <si>
+    <t>Alejandría</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,6 +154,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -179,10 +215,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -600,53 +636,90 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30E1F39A-8C4E-4E16-9851-F4715B1E06E8}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.42578125" style="1"/>
+    <col min="2" max="2" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="1"/>
+    <col min="5" max="5" width="10.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>